<commit_message>
Update Adomo store prices from the new price list
Products take the list's base price; the after-discount price is ignored.
Earlier seeded prices and names are kept in AdomoCatalog.Previous, so a product
is repriced only where it still holds exactly what the earlier version seeded.
The seeder side of this landed in 621af96; this completes it so the committed
tree builds.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/adomo-prices.xlsx
+++ b/docs/adomo-prices.xlsx
@@ -431,14 +431,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="58" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -459,10 +459,15 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>سعر البيع (ر.س)</t>
+          <t>سعر البيع شامل الضريبة (ر.س)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>الحد الأدنى بعد الخصم (ر.س)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ملاحظة</t>
         </is>
@@ -485,11 +490,14 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>40.25</v>
+      </c>
+      <c r="E2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -510,11 +518,14 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>34.5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -535,11 +546,14 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>51</v>
+      </c>
+      <c r="E4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -560,11 +574,14 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>51.75</v>
+      </c>
+      <c r="E5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -585,11 +602,14 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>40.25</v>
+      </c>
+      <c r="E6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -610,11 +630,14 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>34.5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -626,7 +649,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>غسول الوجه الرغوي بجل الصبار 200 مل</t>
+          <t>غسول الوجه الرغوي بجل الصبار والنياسيناميد 200 مل</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -635,11 +658,14 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>60</v>
+      </c>
+      <c r="E8" t="n">
+        <v>16</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -660,11 +686,14 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>57.5</v>
+      </c>
+      <c r="E9" t="n">
+        <v>15</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -685,11 +714,14 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>51.75</v>
+      </c>
+      <c r="E10" t="n">
+        <v>15</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -710,11 +742,14 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>34.75</v>
+      </c>
+      <c r="E11" t="n">
+        <v>12</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -735,11 +770,14 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>77</v>
+      </c>
+      <c r="E12" t="n">
+        <v>15</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -760,11 +798,14 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>34.5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>12</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -785,11 +826,14 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>17.25</v>
+      </c>
+      <c r="E14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -812,9 +856,9 @@
       <c r="D15" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ليس في قائمة أكتوبر 2026 — سعر افتراضي</t>
         </is>
       </c>
     </row>
@@ -837,9 +881,9 @@
       <c r="D16" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ليس في قائمة أكتوبر 2026 — سعر افتراضي</t>
         </is>
       </c>
     </row>
@@ -862,9 +906,9 @@
       <c r="D17" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ليس في قائمة أكتوبر 2026 — سعر افتراضي</t>
         </is>
       </c>
     </row>
@@ -885,11 +929,14 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>3.45</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -910,11 +957,14 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>28.75</v>
+      </c>
+      <c r="E19" t="n">
+        <v>8</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -935,11 +985,14 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>28.75</v>
+      </c>
+      <c r="E20" t="n">
+        <v>8</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -960,11 +1013,14 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>28.75</v>
+      </c>
+      <c r="E21" t="n">
+        <v>8</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -985,11 +1041,14 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>34.5</v>
+      </c>
+      <c r="E22" t="n">
+        <v>12</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -1010,11 +1069,14 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>34.5</v>
+      </c>
+      <c r="E23" t="n">
+        <v>12</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
         </is>
       </c>
     </row>
@@ -1035,11 +1097,70 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>سعر افتراضي — عدّله من لوحة التحكم</t>
+        <v>34.5</v>
+      </c>
+      <c r="E24" t="n">
+        <v>12</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>AD-24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>جل الجلسرين 60 مل</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>العناية بالبشرة</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026 — صورة مؤقتة</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>AD-25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>بلسم الشعر 290 مل</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>العناية بالشعر</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="E26" t="n">
+        <v>12</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>قائمة أسعار ADOMO أكتوبر 2026 — صورة مؤقتة</t>
         </is>
       </c>
     </row>

</xml_diff>